<commit_message>
New Teams and last year prices
</commit_message>
<xml_diff>
--- a/KCC Tournament Season #5 (Responses).xlsx
+++ b/KCC Tournament Season #5 (Responses).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="247">
   <si>
     <t>Timestamp</t>
   </si>
@@ -187,7 +187,7 @@
     <t>https://drive.google.com/open?id=1dVmh-Eo0p6qi-LDyB3DsPZMSkICa6KJq</t>
   </si>
   <si>
-    <t>+91 70584 82858</t>
+    <t xml:space="preserve">                  70584 82858</t>
   </si>
   <si>
     <t>https://drive.google.com/open?id=1Z_0NWRg4FPQYYSFRrVOX1K828WwGhnLC</t>
@@ -505,9 +505,6 @@
     <t>https://drive.google.com/open?id=12CSNnGK0H3ocCMVmbl4NuXyFCLk8UULL</t>
   </si>
   <si>
-    <t>96072 05470</t>
-  </si>
-  <si>
     <t>https://drive.google.com/open?id=1MYmU7q7rckj8i3UgWgfQEMcyWUM-DrW1</t>
   </si>
   <si>
@@ -659,6 +656,102 @@
   </si>
   <si>
     <t>https://drive.google.com/open?id=1c0_BbZPSkHuUwxB2BWhbehih6V9KD0i5</t>
+  </si>
+  <si>
+    <t>Dharmesh jain</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1xdrXjfM9MwrWLAb_iHKBzngvmWpUPjBk</t>
+  </si>
+  <si>
+    <t>+91 95119 10477</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=14g_DbzcyT4Sm9tzy2-e1rnjfpAirOQTS</t>
+  </si>
+  <si>
+    <t>Prem Sancheti</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1EXyflwbyPMyIkgR8w2Oe91duh5WAd98-</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1ELkurnMnChBdNmziyovQ8KL40BLqeisb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shailesh chhajed </t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1_pk9oHHrKwiV_KqYzFIJPuNzCZQD5OGq</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1ty9x0vDINZIHOKuD9PYZhkIIVVe0xAoj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vinay garg </t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1y1Zbex6lMoo_XwH7H1w8LZB0jPuaDvhD</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1GrbhNzVFrXZJD42-TRUpVcf5wxlSkAO1</t>
+  </si>
+  <si>
+    <t>Mahaveer vinod oswal</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1Jd7oxYE6Xap-8HVayup6BnwSdiH9BSoG</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1uUV84q49Uab-Yy-FAENv-dohj5MLGaVg</t>
+  </si>
+  <si>
+    <t>Abhay Ramesh Bhonde</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1CzxS4P3EdOO2_-BLziecCsxhyE3KHs3z</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1M9RrupuBtmSqLclnhr0GSP6bBR7Y48T4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nikhil Bhalgat </t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1NPXBeTsx3dhqRPVSFh60T1XId06aynOq</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1TJiSgr6gngx8kXBCX1_a3tBFo92pDFWW</t>
+  </si>
+  <si>
+    <t>Rushil oswal</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1GRNALFYrVMDUp1XT6Q1wGDkAU0GpEMzG</t>
+  </si>
+  <si>
+    <t>Wicket Keeper</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1GmIkgtzCeRTIla-bc578TZy5r0WWPjyv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balaji Tatewar </t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1E3uLh2bnc8ghlkfF6iegNo8C6SCapj9t</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1PLkUsr7GbwD19JjdLK4ZDo5kxHk2i5W3</t>
+  </si>
+  <si>
+    <t>Arham Darda</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=16MS30LhSI5iyjUP-qmwSgwRU_t6HnvxC</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1RsQxvTlazHNmy21jJqGnY5AE7iC44sFw</t>
   </si>
 </sst>
 </file>
@@ -805,7 +898,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:K65" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:K75" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="11">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Player Name" id="2"/>
@@ -1020,6 +1113,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
+    <tabColor rgb="FF00FF00"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
@@ -2689,8 +2783,8 @@
       <c r="C48" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="D48" s="3" t="s">
-        <v>164</v>
+      <c r="D48" s="3">
+        <v>9.60720547E9</v>
       </c>
       <c r="E48" s="3">
         <v>27.0</v>
@@ -2708,7 +2802,7 @@
         <v>15</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K48" s="3" t="s">
         <v>82</v>
@@ -2719,10 +2813,10 @@
         <v>46024.67186475694</v>
       </c>
       <c r="B49" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C49" s="4" t="s">
         <v>166</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>167</v>
       </c>
       <c r="D49" s="3">
         <v>7.709720539E9</v>
@@ -2743,7 +2837,7 @@
         <v>15</v>
       </c>
       <c r="J49" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K49" s="3" t="s">
         <v>17</v>
@@ -2754,10 +2848,10 @@
         <v>46024.67737914352</v>
       </c>
       <c r="B50" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C50" s="4" t="s">
         <v>169</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>170</v>
       </c>
       <c r="D50" s="3">
         <v>9.172811523E9</v>
@@ -2778,7 +2872,7 @@
         <v>15</v>
       </c>
       <c r="J50" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="K50" s="3" t="s">
         <v>82</v>
@@ -2789,10 +2883,10 @@
         <v>46024.68131545139</v>
       </c>
       <c r="B51" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="C51" s="4" t="s">
         <v>172</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>173</v>
       </c>
       <c r="D51" s="3">
         <v>9.766239953E9</v>
@@ -2813,7 +2907,7 @@
         <v>15</v>
       </c>
       <c r="J51" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K51" s="3" t="s">
         <v>17</v>
@@ -2824,10 +2918,10 @@
         <v>46024.693732291664</v>
       </c>
       <c r="B52" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="C52" s="4" t="s">
         <v>175</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>176</v>
       </c>
       <c r="D52" s="3">
         <v>7.020792596E9</v>
@@ -2848,7 +2942,7 @@
         <v>15</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K52" s="3" t="s">
         <v>82</v>
@@ -2859,10 +2953,10 @@
         <v>46024.7049277662</v>
       </c>
       <c r="B53" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="C53" s="4" t="s">
         <v>178</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>179</v>
       </c>
       <c r="D53" s="3">
         <v>7.330910611E9</v>
@@ -2883,7 +2977,7 @@
         <v>15</v>
       </c>
       <c r="J53" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="K53" s="3" t="s">
         <v>36</v>
@@ -2894,10 +2988,10 @@
         <v>46024.70978217592</v>
       </c>
       <c r="B54" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="C54" s="4" t="s">
         <v>181</v>
-      </c>
-      <c r="C54" s="4" t="s">
-        <v>182</v>
       </c>
       <c r="D54" s="3">
         <v>9.16884311E9</v>
@@ -2918,7 +3012,7 @@
         <v>15</v>
       </c>
       <c r="J54" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K54" s="3" t="s">
         <v>60</v>
@@ -2929,10 +3023,10 @@
         <v>46024.74435028935</v>
       </c>
       <c r="B55" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="C55" s="4" t="s">
         <v>184</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>185</v>
       </c>
       <c r="D55" s="3">
         <v>8.975164636E9</v>
@@ -2953,7 +3047,7 @@
         <v>15</v>
       </c>
       <c r="J55" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="K55" s="3" t="s">
         <v>36</v>
@@ -2964,10 +3058,10 @@
         <v>46024.75057347222</v>
       </c>
       <c r="B56" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="C56" s="4" t="s">
         <v>187</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>188</v>
       </c>
       <c r="D56" s="3">
         <v>7.709947611E9</v>
@@ -2988,7 +3082,7 @@
         <v>15</v>
       </c>
       <c r="J56" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K56" s="3" t="s">
         <v>36</v>
@@ -2999,10 +3093,10 @@
         <v>46024.755376597226</v>
       </c>
       <c r="B57" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C57" s="4" t="s">
         <v>190</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>191</v>
       </c>
       <c r="D57" s="3">
         <v>9.623323445E9</v>
@@ -3023,7 +3117,7 @@
         <v>15</v>
       </c>
       <c r="J57" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="K57" s="3" t="s">
         <v>36</v>
@@ -3034,10 +3128,10 @@
         <v>46024.75677003472</v>
       </c>
       <c r="B58" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="C58" s="4" t="s">
         <v>193</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>194</v>
       </c>
       <c r="D58" s="3">
         <v>9.011239601E9</v>
@@ -3058,7 +3152,7 @@
         <v>15</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="K58" s="3" t="s">
         <v>36</v>
@@ -3069,10 +3163,10 @@
         <v>46024.80902835648</v>
       </c>
       <c r="B59" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="C59" s="7" t="s">
         <v>196</v>
-      </c>
-      <c r="C59" s="7" t="s">
-        <v>197</v>
       </c>
       <c r="D59" s="6">
         <v>7.057175718E9</v>
@@ -3093,7 +3187,7 @@
         <v>15</v>
       </c>
       <c r="J59" s="7" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K59" s="6" t="s">
         <v>60</v>
@@ -3104,10 +3198,10 @@
         <v>46024.83714920139</v>
       </c>
       <c r="B60" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C60" s="7" t="s">
         <v>199</v>
-      </c>
-      <c r="C60" s="7" t="s">
-        <v>200</v>
       </c>
       <c r="D60" s="6">
         <v>8.66852134E9</v>
@@ -3128,7 +3222,7 @@
         <v>15</v>
       </c>
       <c r="J60" s="7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="K60" s="6" t="s">
         <v>17</v>
@@ -3139,10 +3233,10 @@
         <v>46024.87600872685</v>
       </c>
       <c r="B61" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="C61" s="7" t="s">
         <v>202</v>
-      </c>
-      <c r="C61" s="7" t="s">
-        <v>203</v>
       </c>
       <c r="D61" s="6">
         <v>9.607901555E9</v>
@@ -3163,7 +3257,7 @@
         <v>15</v>
       </c>
       <c r="J61" s="7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K61" s="6" t="s">
         <v>82</v>
@@ -3174,10 +3268,10 @@
         <v>46024.91378831019</v>
       </c>
       <c r="B62" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C62" s="7" t="s">
         <v>205</v>
-      </c>
-      <c r="C62" s="7" t="s">
-        <v>206</v>
       </c>
       <c r="D62" s="6">
         <v>9.8221431E9</v>
@@ -3198,7 +3292,7 @@
         <v>15</v>
       </c>
       <c r="J62" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K62" s="6" t="s">
         <v>82</v>
@@ -3212,7 +3306,7 @@
         <v>150</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D63" s="6">
         <v>8.530323363E9</v>
@@ -3233,7 +3327,7 @@
         <v>15</v>
       </c>
       <c r="J63" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="K63" s="6" t="s">
         <v>131</v>
@@ -3244,10 +3338,10 @@
         <v>46025.00984458333</v>
       </c>
       <c r="B64" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="C64" s="7" t="s">
         <v>210</v>
-      </c>
-      <c r="C64" s="7" t="s">
-        <v>211</v>
       </c>
       <c r="D64" s="6">
         <v>8.421732939E9</v>
@@ -3268,7 +3362,7 @@
         <v>15</v>
       </c>
       <c r="J64" s="7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="K64" s="6" t="s">
         <v>60</v>
@@ -3279,10 +3373,10 @@
         <v>46025.52965505787</v>
       </c>
       <c r="B65" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="C65" s="7" t="s">
         <v>213</v>
-      </c>
-      <c r="C65" s="7" t="s">
-        <v>214</v>
       </c>
       <c r="D65" s="6">
         <v>8.688455058E9</v>
@@ -3303,10 +3397,360 @@
         <v>15</v>
       </c>
       <c r="J65" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K65" s="6" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="66" ht="22.5" customHeight="1">
+      <c r="A66" s="5">
+        <v>46025.566172430554</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="E66" s="6">
+        <v>44.0</v>
+      </c>
+      <c r="F66" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G66" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H66" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="I66" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J66" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="K66" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="67" ht="22.5" customHeight="1">
+      <c r="A67" s="5">
+        <v>46025.73952623842</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="C67" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="D67" s="6">
+        <v>9.766324097E9</v>
+      </c>
+      <c r="E67" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G67" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H67" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="I67" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J67" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="K67" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="68" ht="22.5" customHeight="1">
+      <c r="A68" s="5">
+        <v>46025.870082187495</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="C68" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="D68" s="6">
+        <v>9.767036398E9</v>
+      </c>
+      <c r="E68" s="6">
+        <v>44.0</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G68" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H68" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I68" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J68" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="K68" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="69" ht="22.5" customHeight="1">
+      <c r="A69" s="5">
+        <v>46025.871465358796</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="C69" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="D69" s="6">
+        <v>9.767036398E9</v>
+      </c>
+      <c r="E69" s="6">
+        <v>44.0</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G69" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H69" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I69" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J69" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="K69" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="70" ht="22.5" customHeight="1">
+      <c r="A70" s="5">
+        <v>46026.47902755787</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="C70" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="D70" s="6">
+        <v>9.325886507E9</v>
+      </c>
+      <c r="E70" s="6">
+        <v>23.0</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G70" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H70" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I70" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J70" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="K70" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="71" ht="22.5" customHeight="1">
+      <c r="A71" s="5">
+        <v>46026.52785854167</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="C71" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="D71" s="6">
+        <v>9.067064655E9</v>
+      </c>
+      <c r="E71" s="6">
+        <v>25.0</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G71" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H71" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I71" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J71" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="K71" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="72" ht="22.5" customHeight="1">
+      <c r="A72" s="5">
+        <v>46027.47943678241</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="C72" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="D72" s="6">
+        <v>8.149181081E9</v>
+      </c>
+      <c r="E72" s="6">
+        <v>35.0</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G72" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H72" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I72" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J72" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="K72" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="73" ht="22.5" customHeight="1">
+      <c r="A73" s="5">
+        <v>46027.53183309028</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C73" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="D73" s="6">
+        <v>9.834718577E9</v>
+      </c>
+      <c r="E73" s="6">
+        <v>27.0</v>
+      </c>
+      <c r="F73" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G73" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H73" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="I73" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J73" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="K73" s="6" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="74" ht="22.5" customHeight="1">
+      <c r="A74" s="5">
+        <v>46027.82061123842</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="C74" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D74" s="6">
+        <v>7.88782828E9</v>
+      </c>
+      <c r="E74" s="6">
+        <v>39.0</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G74" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H74" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I74" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J74" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="K74" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="75" ht="22.5" customHeight="1">
+      <c r="A75" s="5">
+        <v>46027.86993271991</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="C75" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="D75" s="6">
+        <v>8.805332992E9</v>
+      </c>
+      <c r="E75" s="6">
+        <v>17.0</v>
+      </c>
+      <c r="F75" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G75" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H75" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="I75" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J75" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="K75" s="6" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -3439,10 +3883,30 @@
     <hyperlink r:id="rId126" ref="J64"/>
     <hyperlink r:id="rId127" ref="C65"/>
     <hyperlink r:id="rId128" ref="J65"/>
+    <hyperlink r:id="rId129" ref="C66"/>
+    <hyperlink r:id="rId130" ref="J66"/>
+    <hyperlink r:id="rId131" ref="C67"/>
+    <hyperlink r:id="rId132" ref="J67"/>
+    <hyperlink r:id="rId133" ref="C68"/>
+    <hyperlink r:id="rId134" ref="J68"/>
+    <hyperlink r:id="rId135" ref="C69"/>
+    <hyperlink r:id="rId136" ref="J69"/>
+    <hyperlink r:id="rId137" ref="C70"/>
+    <hyperlink r:id="rId138" ref="J70"/>
+    <hyperlink r:id="rId139" ref="C71"/>
+    <hyperlink r:id="rId140" ref="J71"/>
+    <hyperlink r:id="rId141" ref="C72"/>
+    <hyperlink r:id="rId142" ref="J72"/>
+    <hyperlink r:id="rId143" ref="C73"/>
+    <hyperlink r:id="rId144" ref="J73"/>
+    <hyperlink r:id="rId145" ref="C74"/>
+    <hyperlink r:id="rId146" ref="J74"/>
+    <hyperlink r:id="rId147" ref="C75"/>
+    <hyperlink r:id="rId148" ref="J75"/>
   </hyperlinks>
-  <drawing r:id="rId129"/>
+  <drawing r:id="rId149"/>
   <tableParts count="1">
-    <tablePart r:id="rId131"/>
+    <tablePart r:id="rId151"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>